<commit_message>
feat(fichas): Proyecto Carretera - Granulometria+Atterberg (GRA: tamizado+huso, LL recta de flujo, LP/IP) y CBR (3 moldes, esfuerzo/CBR 0.1-0.2, interpolacion al %DMS via xref al Proctor); aux capas ampliada (CBR/PctDMS/Exp/LL/IP); validado con el motor
</commit_message>
<xml_diff>
--- a/Proyectos Modelo/Proyecto_Carretera/Carretera_TablasAuxiliares.xlsx
+++ b/Proyectos Modelo/Proyecto_Carretera/Carretera_TablasAuxiliares.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -450,9 +450,94 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>tabla-capas_pavimento</v>
+      </c>
+      <c r="B4" t="str">
+        <v>CBRmin</v>
+      </c>
+      <c r="C4">
+        <v>80</v>
+      </c>
+      <c r="D4">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>tabla-capas_pavimento</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PctDMS</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5">
+        <v>95</v>
+      </c>
+      <c r="E5">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>tabla-capas_pavimento</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ExpMax</v>
+      </c>
+      <c r="C6">
+        <v>0.5</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>tabla-capas_pavimento</v>
+      </c>
+      <c r="B7" t="str">
+        <v>LLmax</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+      <c r="E7">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>tabla-capas_pavimento</v>
+      </c>
+      <c r="B8" t="str">
+        <v>IPmax</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+      <c r="E8">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>